<commit_message>
Changes as per requirements
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -1,91 +1,99 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automate\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\t\Automate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{341FDAF0-1C1C-4096-BA57-31A8A099B863}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{851CBB04-634B-461D-AE74-4226E099A721}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D3020824-1DB6-4EC1-8847-11B2806A916D}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D3020824-1DB6-4EC1-8847-11B2806A916D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
-  <si>
-    <t>M95A</t>
-  </si>
-  <si>
-    <t>N245N</t>
-  </si>
-  <si>
-    <t>NO.5699</t>
-  </si>
-  <si>
-    <t>IMG-20260313-WA0006</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1E1OLYoD5TznDE7qPgRMCRBvIlWPRHjee/view?usp=sharing</t>
-  </si>
-  <si>
-    <t>Code</t>
-  </si>
-  <si>
-    <t>other code</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>original price Rs. (A)</t>
   </si>
   <si>
-    <t xml:space="preserve">35%Margin price Rs </t>
-  </si>
-  <si>
     <t>Roud Off (B)</t>
   </si>
   <si>
-    <t>(Our Price Rs (A +B)</t>
-  </si>
-  <si>
     <t>File Name</t>
   </si>
   <si>
     <t>Drive Link</t>
   </si>
   <si>
-    <t xml:space="preserve">Original Item Description </t>
-  </si>
-  <si>
-    <t>*Micro Gold Mangalsutra Set* Length- 38Inch Price -490rs FREE SHIPPING ALL OVER INDIA😊</t>
-  </si>
-  <si>
-    <t>*Micro Gold Mangalsutra Set* Length- 38Inch Price - 662 FREE SHIPPING ALL OVER INDIA😊</t>
-  </si>
-  <si>
     <t>Modified Item Description</t>
+  </si>
+  <si>
+    <t>Original Item Description</t>
+  </si>
+  <si>
+    <t>35%Margin price Rs</t>
+  </si>
+  <si>
+    <t>Extracted Codes (OCR)</t>
+  </si>
+  <si>
+    <t>IMG-20260310-WA0002.jpg</t>
+  </si>
+  <si>
+    <t>*New Micro Gold  Mangalsutra Combo set* Length- 34Inch Price -540rs FREE SHIPPING ALL OVER INDIA😊</t>
+  </si>
+  <si>
+    <t>Code-1110, SAC, M1O4B, N2ZON, 7810044, 8919534, No.3800, 5 A, L34 inch</t>
+  </si>
+  <si>
+    <t>VID-20260319-WA0044.mp4</t>
+  </si>
+  <si>
+    <t>**1 GM FORMING MAHARAJ KADA* ( Half Kada Adjustable ) Price - 470 rs Each *FREE SHIPPING ALL OVER INDIA😊*</t>
+  </si>
+  <si>
+    <t>Code-827, A'C, M9OB, N235N, 8325067, No.9600, 1GM Forming</t>
+  </si>
+  <si>
+    <t>IMG-20260310-WA0005.jpg</t>
+  </si>
+  <si>
+    <t>*1 GM FORMING श्री स्वामी समर्थ CHAIN* Length- 24Inch Price -450rs FREE SHIPPING ALL OVER INDIA😊</t>
+  </si>
+  <si>
+    <t>*1 GM FORMING श्री स्वामी समर्थ CHAIN* Length- 24Inch Price -608rs FREE SHIPPING ALL OVER INDIA😊</t>
+  </si>
+  <si>
+    <t>Code-1161, M86B, N22SN, 8920056, No.6700, CHAIN, L-24 Inch, 7Fef</t>
+  </si>
+  <si>
+    <t>Increaded Price</t>
+  </si>
+  <si>
+    <t>Our Price Rs(Round off to neareast divisible by 5)</t>
+  </si>
+  <si>
+    <t>*New Micro Gold  Mangalsutra Combo set* Length- 34Inch Price -730rs FREE SHIPPING ALL OVER INDIA😊</t>
+  </si>
+  <si>
+    <t>**1 GM FORMING MAHARAJ KADA* ( Half Kada Adjustable ) Price - 635 rs Each *FREE SHIPPING ALL OVER INDIA😊*</t>
+  </si>
+  <si>
+    <t>Date of Message</t>
   </si>
 </sst>
 </file>
@@ -107,10 +115,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -121,10 +128,36 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -133,21 +166,40 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF4C7C3"/>
+          <bgColor rgb="FFF4C7C3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB7E1CD"/>
+          <bgColor rgb="FFB7E1CD"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -474,113 +526,156 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F206FB67-0C86-4FB1-B05B-987632DF1F43}">
-  <dimension ref="A1:R2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:S4"/>
+  <sheetFormatPr defaultColWidth="26.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="8" max="8" width="22.77734375" customWidth="1"/>
+    <col min="4" max="4" width="141" customWidth="1"/>
+    <col min="10" max="10" width="60.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C1" s="1" t="s">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="G1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A2" s="5">
+        <v>46091</v>
+      </c>
+      <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="D2" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="E2">
+        <v>540</v>
+      </c>
+      <c r="F2">
+        <v>189</v>
+      </c>
+      <c r="G2">
+        <v>189</v>
+      </c>
+      <c r="H2">
+        <v>729</v>
+      </c>
+      <c r="I2">
+        <v>730</v>
+      </c>
+      <c r="J2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="1">
-        <v>1157</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F2" s="1">
-        <v>7829056</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" s="1">
-        <v>490</v>
-      </c>
-      <c r="J2" s="1">
-        <f t="shared" ref="J2" si="0">I2*35%</f>
-        <v>171.5</v>
-      </c>
-      <c r="K2" s="1">
-        <f t="shared" ref="K2" si="1">ROUNDUP(J2,0)</f>
-        <v>172</v>
-      </c>
-      <c r="L2" s="1">
-        <f t="shared" ref="L2" si="2">I2+K2</f>
-        <v>662</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
       <c r="P2" s="1"/>
-      <c r="Q2" s="4"/>
-      <c r="R2" s="1"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="1"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A3" s="5">
+        <v>46091</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3">
+        <v>470</v>
+      </c>
+      <c r="F3">
+        <v>164.5</v>
+      </c>
+      <c r="G3">
+        <v>164</v>
+      </c>
+      <c r="H3">
+        <v>634</v>
+      </c>
+      <c r="I3">
+        <v>635</v>
+      </c>
+      <c r="J3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A4" s="5">
+        <v>46091</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4">
+        <v>450</v>
+      </c>
+      <c r="F4">
+        <v>157.5</v>
+      </c>
+      <c r="G4">
+        <v>158</v>
+      </c>
+      <c r="H4">
+        <v>608</v>
+      </c>
+      <c r="I4">
+        <v>610</v>
+      </c>
+      <c r="J4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K4" t="s">
+        <v>17</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="D1:G1"/>
-  </mergeCells>
-  <conditionalFormatting sqref="D1:D2">
-    <cfRule type="expression" dxfId="1" priority="3">
-      <formula>COUNTIF(C:C, C1)&gt;1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F2">
-    <cfRule type="containsBlanks" dxfId="0" priority="4">
-      <formula>LEN(TRIM(F2))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{44D9874B-AF57-4710-96F6-026D888137BA}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>